<commit_message>
Working version with load and NTCs, should be cleaned up before deciding on the question of regional renewables
</commit_message>
<xml_diff>
--- a/input/geo_list_of_nodes - Excel 2.xlsx
+++ b/input/geo_list_of_nodes - Excel 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boissieremat\Documents\GitHub\antares-brinkerink-2015\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FFDD4544-96B5-4F58-B8F7-77DBEBB1A3B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B83D66B-706E-432D-A753-E607C205CD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25320" yWindow="-60" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3864,16 +3864,13 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -3898,6 +3895,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -3964,33 +3964,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6D89E52A-B272-4F51-A5B5-64AFC4B47FBE}" name="geo_list_of_nodes" displayName="geo_list_of_nodes" ref="A1:H266" tableType="queryTable" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6D89E52A-B272-4F51-A5B5-64AFC4B47FBE}" name="geo_list_of_nodes" displayName="geo_list_of_nodes" ref="A1:H266" tableType="queryTable" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A1:H266" xr:uid="{6D89E52A-B272-4F51-A5B5-64AFC4B47FBE}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{284128C1-B1F5-4332-AB15-51820AA94D7B}" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{07E0DCA2-7634-47C6-989B-D9A41A33CD8E}" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{5B30FEED-158C-4351-B6AD-DC0EE31B9A99}" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{22025BB5-F973-40CA-A8DE-05EFFB681C89}" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{FD369853-86F3-4E18-8346-69B0C2E12458}" uniqueName="9" name="node_source" queryTableFieldId="9" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{C634F726-4E37-49C9-87D1-101A99B34B2A}" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{4449F2E7-AA8A-4790-B084-BD642B4EE338}" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{3838D257-94B0-46FF-A191-7A07FF5997FB}" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{284128C1-B1F5-4332-AB15-51820AA94D7B}" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{07E0DCA2-7634-47C6-989B-D9A41A33CD8E}" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{5B30FEED-158C-4351-B6AD-DC0EE31B9A99}" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{22025BB5-F973-40CA-A8DE-05EFFB681C89}" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{FD369853-86F3-4E18-8346-69B0C2E12458}" uniqueName="9" name="node_source" queryTableFieldId="9" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{C634F726-4E37-49C9-87D1-101A99B34B2A}" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{4449F2E7-AA8A-4790-B084-BD642B4EE338}" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{3838D257-94B0-46FF-A191-7A07FF5997FB}" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="geo_list_of_nodes___Excel" displayName="geo_list_of_nodes___Excel" ref="A1:G259" tableType="queryTable" totalsRowShown="0" headerRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="geo_list_of_nodes___Excel" displayName="geo_list_of_nodes___Excel" ref="A1:G259" tableType="queryTable" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="A1:G259" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>